<commit_message>
Ornek sablon Turkce karakterlerle guncellendi
</commit_message>
<xml_diff>
--- a/apps/frontend/public/ornek-urun-sablonu.xlsx
+++ b/apps/frontend/public/ornek-urun-sablonu.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Urun Listesi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Referans Degerler" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ürün Listesi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Referans Değerler" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +29,7 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="00777777"/>
       <sz val="9"/>
     </font>
     <font>
@@ -53,7 +53,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F0F0"/>
+        <fgColor rgb="00F4F4F4"/>
       </patternFill>
     </fill>
     <fill>
@@ -87,16 +87,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00B0C8E0"/>
+        <color rgb="00C0D4E8"/>
       </left>
       <right style="thin">
-        <color rgb="00B0C8E0"/>
+        <color rgb="00C0D4E8"/>
       </right>
       <top style="thin">
-        <color rgb="00B0C8E0"/>
+        <color rgb="00C0D4E8"/>
       </top>
       <bottom style="thin">
-        <color rgb="00B0C8E0"/>
+        <color rgb="00C0D4E8"/>
       </bottom>
     </border>
   </borders>
@@ -494,9 +494,9 @@
   <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -514,99 +514,99 @@
     <col width="24" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="38" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Urun stok kodu (benzersiz)</t>
+          <t>Ürüne özel benzersiz stok kodu</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Urunun tam adi</t>
+          <t>Ürünün tam adı</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Urun tipi (serbest metin)</t>
+          <t>Ürün tipi — serbest metin</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Genislik - cm cinsinden</t>
+          <t>Genişlik (cm)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Uzunluk - cm cinsinden</t>
+          <t>Uzunluk (cm)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Yukseklik - cm cinsinden</t>
+          <t>Yükseklik (cm)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Agirlik - kg cinsinden</t>
+          <t>Ağırlık (kg)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>NonFragile/Fragile/LiquidChemical/Flammable/Oxidizing</t>
+          <t>Kırılmaz / Kırılgan / Sıvı Kimyasal / Yanıcı / Oksitleyici</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>evet veya hayir</t>
+          <t>evet veya hayır</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Istiflenebilir=evet ise zorunlu (&gt;0)</t>
+          <t>İstiflenebilir=evet ise zorunlu, 0'dan büyük olmalı</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Istiflenebilir=evet ise zorunlu, kg (&gt;0)</t>
+          <t>İstiflenebilir=evet ise zorunlu, 0'dan büyük olmalı (kg)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Barkod numarasi (opsiyonel)</t>
+          <t>Barkod numarası (opsiyonel)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Package / Pallet / Box (varsayilan: Package)</t>
+          <t>Paket / Palet / Kutu  (varsayılan: Paket)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Silindirik urunler icin cap - cm (opsiyonel)</t>
+          <t>Silindirik ürünler için çap, cm (opsiyonel)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>All / NoVertical / Fixed (varsayilan: All)</t>
+          <t>Tümü / Dikey Yok / Sabit  (varsayılan: Tümü)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Urun resmi URL (opsiyonel)</t>
+          <t>Ürün resmi adresi (opsiyonel)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Istif grubu kodu (opsiyonel)</t>
+          <t>İstif grubu kodu (opsiyonel)</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Serbest not alani (opsiyonel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
+          <t>Serbest not alanı (opsiyonel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>SKU</t>
@@ -614,12 +614,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Urun Adi</t>
+          <t>Ürün Adı</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Urun Tipi</t>
+          <t>Ürün Tipi</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -634,32 +634,32 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Yukseklik</t>
+          <t>Yükseklik</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Agirlik</t>
+          <t>Ağırlık</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Hassasiyet Turu</t>
+          <t>Hassasiyet Türü</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Istiflenebilir</t>
+          <t>İstiflenebilir</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>Max Istif Sayisi</t>
+          <t>Max İstif Sayısı</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Max Agirlik Ustunde</t>
+          <t>Max Ağırlık Üstünde</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -674,12 +674,12 @@
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>Cap</t>
+          <t>Çap</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>Izin Verilen Rotasyonlar</t>
+          <t>İzin Verilen Rotasyonlar</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
@@ -689,71 +689,63 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>Istif Grubu</t>
+          <t>İstif Grubu</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>Ozel Notlar</t>
+          <t>Özel Notlar</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>SKU-001</t>
+          <t>LPT-ACER-001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Tasima Kolisi A</t>
+          <t>Acer Nitro 5 Laptop</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Standart Koli</t>
+          <t>Elektronik</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>36.3</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>25.5</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>2.4</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>NonFragile</t>
+          <t>Kırılgan</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>evet</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
+          <t>hayır</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
           <t>8691234567890</t>
@@ -761,13 +753,13 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>Package</t>
+          <t>Paket</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr"/>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Tümü</t>
         </is>
       </c>
       <c r="P3" s="4" t="inlineStr"/>
@@ -789,8 +781,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -801,97 +793,97 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Deger</t>
+          <t>Excel'e Yazılacak Değer</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Aciklama</t>
+          <t>Açıklama</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Hassasiyet Turu</t>
+          <t>Hassasiyet Türü</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>NonFragile</t>
+          <t>Kırılmaz</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Kirigan degil</t>
+          <t>NonFragile — kırılmaz, sağlam ürün</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Hassasiyet Turu</t>
+          <t>Hassasiyet Türü</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Fragile</t>
+          <t>Kırılgan</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Kirigan</t>
+          <t>Fragile — dikkatli taşınması gereken ürün</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Hassasiyet Turu</t>
+          <t>Hassasiyet Türü</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>LiquidChemical</t>
+          <t>Sıvı Kimyasal</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Sivi / Kimyasal</t>
+          <t>LiquidChemical — sıvı veya kimyasal madde</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Hassasiyet Turu</t>
+          <t>Hassasiyet Türü</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Flammable</t>
+          <t>Yanıcı</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Yanici</t>
+          <t>Flammable — yanıcı madde</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Hassasiyet Turu</t>
+          <t>Hassasiyet Türü</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Oxidizing</t>
+          <t>Oksitleyici</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Oksitleyici</t>
+          <t>Oxidizing — oksitleyici madde</t>
         </is>
       </c>
     </row>
@@ -908,12 +900,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Package</t>
+          <t>Paket</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Paket (varsayilan)</t>
+          <t>Package — genel paket (varsayılan)</t>
         </is>
       </c>
     </row>
@@ -925,12 +917,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Pallet</t>
+          <t>Palet</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Palet</t>
+          <t>Pallet — palet üzeri ürün</t>
         </is>
       </c>
     </row>
@@ -942,12 +934,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>Kutu</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Kutu</t>
+          <t>Box — kutu</t>
         </is>
       </c>
     </row>
@@ -959,51 +951,51 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Izin Verilen Rotasyonlar</t>
+          <t>İzin Verilen Rotasyonlar</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Tümü</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Tum rotasyonlar serbest (varsayilan)</t>
+          <t>All — tüm yönlere döndürülebilir (varsayılan)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Izin Verilen Rotasyonlar</t>
+          <t>İzin Verilen Rotasyonlar</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>NoVertical</t>
+          <t>Dikey Yok</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Dikey rotasyon yasak</t>
+          <t>NoVertical — dikey rotasyon yapılamaz</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Izin Verilen Rotasyonlar</t>
+          <t>İzin Verilen Rotasyonlar</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Sabit</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Rotasyon yasak</t>
+          <t>Fixed — hiç döndürülemez</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1007,7 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Istiflenebilir</t>
+          <t>İstiflenebilir</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -1025,24 +1017,24 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Istiflenebilir (true/1/yes de kabul edilir)</t>
+          <t>Üstüne başka ürün istiflenebilir</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Istiflenebilir</t>
+          <t>İstiflenebilir</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>hayir</t>
+          <t>hayır</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Istifilenemez (false/0/no de kabul edilir)</t>
+          <t>Üstüne ürün istiflenmez</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ornek sablon genel urunle guncellendi
</commit_message>
<xml_diff>
--- a/apps/frontend/public/ornek-urun-sablonu.xlsx
+++ b/apps/frontend/public/ornek-urun-sablonu.xlsx
@@ -701,54 +701,62 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>LPT-ACER-001</t>
+          <t>ORNEK-001</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Acer Nitro 5 Laptop</t>
+          <t>Örnek Ürün</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Elektronik</t>
+          <t>Genel Ürün</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>36.3</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>25.5</t>
+          <t>40</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>20</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Kırılgan</t>
+          <t>Kırılmaz</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>hayır</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr"/>
-      <c r="K3" s="4" t="inlineStr"/>
+          <t>evet</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>8691234567890</t>
+          <t>1234567890123</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">

</xml_diff>